<commit_message>
Build site at 2021-05-10 20:06:24 UTC
</commit_message>
<xml_diff>
--- a/_scripts/Publicacoes.xlsx
+++ b/_scripts/Publicacoes.xlsx
@@ -19,12 +19,18 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="4" count="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="6" count="6">
   <si>
-    <t>10.1007/978-3-319-19443-1_24</t>
+    <t>Duplicate?</t>
+  </si>
+  <si>
+    <t>no</t>
   </si>
   <si>
     <t>10.1016/j.calphad.2019.101676</t>
+  </si>
+  <si>
+    <t>yes</t>
   </si>
   <si>
     <t>10.1016/j.jallcom.2019.06.186</t>
@@ -153,6 +159,9 @@
           <t>DOI</t>
         </is>
       </c>
+      <c r="B1" s="2" t="s">
+        <v>0</v>
+      </c>
     </row>
     <row r="2" spans="1:16384" customHeight="1" ht="15.75">
       <c r="A2" s="3" t="inlineStr">
@@ -160,19 +169,21 @@
           <t>10.1002/3527607285.ch54</t>
         </is>
       </c>
-      <c r="B2" s="3">
-        <f>COUNTIF(A:A,"="&amp;A2)</f>
+      <c r="B2" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A2)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="4"/>
     </row>
     <row r="3" spans="1:16384" customHeight="1" ht="15.75">
-      <c r="A3" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="3">
-        <f>COUNTIF(A:A,"="&amp;A3)</f>
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>10.1007/978-3-319-19443-1_24</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A3)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="C3" s="3"/>
@@ -184,8 +195,8 @@
           <t>10.1007/BF0273644</t>
         </is>
       </c>
-      <c r="B4" s="3">
-        <f>COUNTIF(A:A,"="&amp;A4)</f>
+      <c r="B4" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A4)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="C4" s="3"/>
@@ -197,8 +208,8 @@
           <t>10.1007/s11085-014-9517-0</t>
         </is>
       </c>
-      <c r="B5" s="3">
-        <f>COUNTIF(A:A,"="&amp;A5)</f>
+      <c r="B5" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A5)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="C5" s="3"/>
@@ -210,8 +221,8 @@
           <t>10.1007/s11085-020-10013-8</t>
         </is>
       </c>
-      <c r="B6" s="3">
-        <f>COUNTIF(A:A,"="&amp;A6)</f>
+      <c r="B6" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A6)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="C6" s="3"/>
@@ -223,8 +234,8 @@
           <t>10.1007/s11661-013-1607-0</t>
         </is>
       </c>
-      <c r="B7" s="3">
-        <f>COUNTIF(A:A,"="&amp;A7)</f>
+      <c r="B7" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A7)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="C7" s="3"/>
@@ -236,8 +247,8 @@
           <t>10.1007/s11661-021-06252-2</t>
         </is>
       </c>
-      <c r="B8" s="3">
-        <f>COUNTIF(A:A,"="&amp;A8)</f>
+      <c r="B8" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A8)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="C8" s="3"/>
@@ -249,8 +260,8 @@
           <t>10.1007/s11665-013-0531-1</t>
         </is>
       </c>
-      <c r="B9" s="3">
-        <f>COUNTIF(A:A,"="&amp;A9)</f>
+      <c r="B9" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A9)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="C9" s="3"/>
@@ -262,8 +273,8 @@
           <t>10.1007/s11665-013-0565-4</t>
         </is>
       </c>
-      <c r="B10" s="3">
-        <f>COUNTIF(A:A,"="&amp;A10)</f>
+      <c r="B10" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A10)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="C10" s="3"/>
@@ -275,8 +286,8 @@
           <t>10.1007/s11665-013-0814-6</t>
         </is>
       </c>
-      <c r="B11" s="3">
-        <f>COUNTIF(A:A,"="&amp;A11)</f>
+      <c r="B11" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A11)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="C11" s="3"/>
@@ -288,8 +299,8 @@
           <t>10.1007/s11665-016-2051-2</t>
         </is>
       </c>
-      <c r="B12" s="3">
-        <f>COUNTIF(A:A,"="&amp;A12)</f>
+      <c r="B12" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A12)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="C12" s="3"/>
@@ -301,8 +312,8 @@
           <t>10.1007/s11665-016-2462-0</t>
         </is>
       </c>
-      <c r="B13" s="3">
-        <f>COUNTIF(A:A,"="&amp;A13)</f>
+      <c r="B13" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A13)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="C13" s="3"/>
@@ -314,8 +325,8 @@
           <t>10.1007/s11665-018-3699-6</t>
         </is>
       </c>
-      <c r="B14" s="3">
-        <f>COUNTIF(A:A,"="&amp;A14)</f>
+      <c r="B14" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A14)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="C14" s="3"/>
@@ -327,8 +338,8 @@
           <t>10.1007/s11665-019-04014-1</t>
         </is>
       </c>
-      <c r="B15" s="3">
-        <f>COUNTIF(A:A,"="&amp;A15)</f>
+      <c r="B15" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A15)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="C15" s="3"/>
@@ -340,8 +351,8 @@
           <t>10.1007/s11669-001-0074-2</t>
         </is>
       </c>
-      <c r="B16" s="3">
-        <f>COUNTIF(A:A,"="&amp;A16)</f>
+      <c r="B16" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A16)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="C16" s="3"/>
@@ -353,8 +364,8 @@
           <t>10.1007/s11669-004-0006-z</t>
         </is>
       </c>
-      <c r="B17" s="3">
-        <f>COUNTIF(A:A,"="&amp;A17)</f>
+      <c r="B17" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A17)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="C17" s="3"/>
@@ -366,8 +377,8 @@
           <t>10.1007/s11669-008-9390-0</t>
         </is>
       </c>
-      <c r="B18" s="3">
-        <f>COUNTIF(A:A,"="&amp;A18)</f>
+      <c r="B18" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A18)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="C18" s="3"/>
@@ -379,8 +390,8 @@
           <t>10.1007/s11669-009-9533-y</t>
         </is>
       </c>
-      <c r="B19" s="3">
-        <f>COUNTIF(A:A,"="&amp;A19)</f>
+      <c r="B19" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A19)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="C19" s="3"/>
@@ -392,8 +403,8 @@
           <t>10.1007/s11669-009-9610-2</t>
         </is>
       </c>
-      <c r="B20" s="3">
-        <f>COUNTIF(A:A,"="&amp;A20)</f>
+      <c r="B20" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A20)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="C20" s="3"/>
@@ -405,8 +416,8 @@
           <t>10.1007/s11669-010-9846-x</t>
         </is>
       </c>
-      <c r="B21" s="3">
-        <f>COUNTIF(A:A,"="&amp;A21)</f>
+      <c r="B21" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A21)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="C21" s="3"/>
@@ -418,8 +429,8 @@
           <t>10.1007/s11669-014-0330-x</t>
         </is>
       </c>
-      <c r="B22" s="3">
-        <f>COUNTIF(A:A,"="&amp;A22)</f>
+      <c r="B22" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A22)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="C22" s="3"/>
@@ -431,8 +442,8 @@
           <t>10.1007/s11669-015-0374-6</t>
         </is>
       </c>
-      <c r="B23" s="3">
-        <f>COUNTIF(A:A,"="&amp;A23)</f>
+      <c r="B23" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A23)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="C23" s="3"/>
@@ -444,8 +455,8 @@
           <t>10.1007/s11669-015-0418-y</t>
         </is>
       </c>
-      <c r="B24" s="3">
-        <f>COUNTIF(A:A,"="&amp;A24)</f>
+      <c r="B24" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A24)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC24" s="0"/>
@@ -457,8 +468,8 @@
           <t>10.1007/s11669-019-00756-6</t>
         </is>
       </c>
-      <c r="B25" s="3">
-        <f>COUNTIF(A:A,"="&amp;A25)</f>
+      <c r="B25" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A25)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC25" s="0"/>
@@ -470,8 +481,8 @@
           <t>10.1007/s11669-020-00787-4</t>
         </is>
       </c>
-      <c r="B26" s="3">
-        <f>COUNTIF(A:A,"="&amp;A26)</f>
+      <c r="B26" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A26)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC26" s="0"/>
@@ -483,8 +494,8 @@
           <t>10.1007/s11669-020-00802-8</t>
         </is>
       </c>
-      <c r="B27" s="3">
-        <f>COUNTIF(A:A,"="&amp;A27)</f>
+      <c r="B27" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A27)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC27" s="0"/>
@@ -496,8 +507,8 @@
           <t>10.1007/s11669-020-00819-z</t>
         </is>
       </c>
-      <c r="B28" s="3">
-        <f>COUNTIF(A:A,"="&amp;A28)</f>
+      <c r="B28" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A28)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC28" s="0"/>
@@ -509,8 +520,8 @@
           <t>10.1007/s11669-020-00838-w</t>
         </is>
       </c>
-      <c r="B29" s="3">
-        <f>COUNTIF(A:A,"="&amp;A29)</f>
+      <c r="B29" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A29)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC29" s="0"/>
@@ -522,8 +533,8 @@
           <t>10.1007/s40430-018-1375-2</t>
         </is>
       </c>
-      <c r="B30" s="3">
-        <f>COUNTIF(A:A,"="&amp;A30)</f>
+      <c r="B30" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A30)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC30" s="0"/>
@@ -535,8 +546,8 @@
           <t>10.1007/s42452-019-1479-z</t>
         </is>
       </c>
-      <c r="B31" s="3">
-        <f>COUNTIF(A:A,"="&amp;A31)</f>
+      <c r="B31" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A31)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC31" s="0"/>
@@ -548,8 +559,8 @@
           <t>10.1016/j.actamat.2005.04.020</t>
         </is>
       </c>
-      <c r="B32" s="3">
-        <f>COUNTIF(A:A,"="&amp;A32)</f>
+      <c r="B32" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A32)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC32" s="0"/>
@@ -561,8 +572,8 @@
           <t>10.1016/j.calphad.2017.10.001</t>
         </is>
       </c>
-      <c r="B33" s="3">
-        <f>COUNTIF(A:A,"="&amp;A33)</f>
+      <c r="B33" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A33)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC33" s="0"/>
@@ -574,8 +585,8 @@
           <t>10.1016/j.calphad.2018.05.004</t>
         </is>
       </c>
-      <c r="B34" s="3">
-        <f>COUNTIF(A:A,"="&amp;A34)</f>
+      <c r="B34" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A34)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC34" s="0"/>
@@ -587,8 +598,8 @@
           <t>10.1016/j.calphad.2018.08.012</t>
         </is>
       </c>
-      <c r="B35" s="3">
-        <f>COUNTIF(A:A,"="&amp;A35)</f>
+      <c r="B35" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A35)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC35" s="0"/>
@@ -596,22 +607,22 @@
     </row>
     <row r="36" spans="1:16384" customHeight="1" ht="15.75">
       <c r="A36" s="0" t="s">
-        <v>1</v>
-      </c>
-      <c r="B36" s="3">
-        <f>COUNTIF(A:A,"="&amp;A36)</f>
         <v>2</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A36)&gt;1,"yes","no")</f>
+        <v>3</v>
       </c>
       <c r="XFC36" s="0"/>
       <c r="XFD36" s="0"/>
     </row>
     <row r="37" spans="1:16384" customHeight="1" ht="15.75">
       <c r="A37" s="0" t="s">
-        <v>1</v>
-      </c>
-      <c r="B37" s="3">
-        <f>COUNTIF(A:A,"="&amp;A37)</f>
         <v>2</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A37)&gt;1,"yes","no")</f>
+        <v>3</v>
       </c>
       <c r="XFC37" s="0"/>
       <c r="XFD37" s="0"/>
@@ -622,8 +633,8 @@
           <t>10.1016/j.calphad.2019.101687</t>
         </is>
       </c>
-      <c r="B38" s="3">
-        <f>COUNTIF(A:A,"="&amp;A38)</f>
+      <c r="B38" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A38)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC38" s="0"/>
@@ -635,8 +646,8 @@
           <t>10.1016/j.calphad.2020.102196</t>
         </is>
       </c>
-      <c r="B39" s="3">
-        <f>COUNTIF(A:A,"="&amp;A39)</f>
+      <c r="B39" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A39)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC39" s="0"/>
@@ -648,8 +659,8 @@
           <t>10.1016/j.ceramint.2020.11.013</t>
         </is>
       </c>
-      <c r="B40" s="3">
-        <f>COUNTIF(A:A,"="&amp;A40)</f>
+      <c r="B40" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A40)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC40" s="0"/>
@@ -661,8 +672,8 @@
           <t>10.1016/j.corsci.2019.108165</t>
         </is>
       </c>
-      <c r="B41" s="3">
-        <f>COUNTIF(A:A,"="&amp;A41)</f>
+      <c r="B41" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A41)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC41" s="0"/>
@@ -674,8 +685,8 @@
           <t>10.1016/j.ijrmhm.2005.06.001</t>
         </is>
       </c>
-      <c r="B42" s="3">
-        <f>COUNTIF(A:A,"="&amp;A42)</f>
+      <c r="B42" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A42)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC42" s="0"/>
@@ -687,8 +698,8 @@
           <t>10.1016/j.ijrmhm.2010.09.006</t>
         </is>
       </c>
-      <c r="B43" s="3">
-        <f>COUNTIF(A:A,"="&amp;A43)</f>
+      <c r="B43" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A43)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC43" s="0"/>
@@ -700,8 +711,8 @@
           <t>10.1016/j.ijrmhm.2011.06.012</t>
         </is>
       </c>
-      <c r="B44" s="3">
-        <f>COUNTIF(A:A,"="&amp;A44)</f>
+      <c r="B44" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A44)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC44" s="0"/>
@@ -713,8 +724,8 @@
           <t>10.1016/j.ijrmhm.2012.04.008</t>
         </is>
       </c>
-      <c r="B45" s="3">
-        <f>COUNTIF(A:A,"="&amp;A45)</f>
+      <c r="B45" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A45)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC45" s="0"/>
@@ -726,8 +737,8 @@
           <t>10.1016/j.intermet.2003.09.015</t>
         </is>
       </c>
-      <c r="B46" s="3">
-        <f>COUNTIF(A:A,"="&amp;A46)</f>
+      <c r="B46" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A46)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC46" s="0"/>
@@ -739,8 +750,8 @@
           <t>10.1016/j.intermet.2004.01.001</t>
         </is>
       </c>
-      <c r="B47" s="3">
-        <f>COUNTIF(A:A,"="&amp;A47)</f>
+      <c r="B47" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A47)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC47" s="0"/>
@@ -752,8 +763,8 @@
           <t>10.1016/j.intermet.2005.05.007</t>
         </is>
       </c>
-      <c r="B48" s="3">
-        <f>COUNTIF(A:A,"="&amp;A48)</f>
+      <c r="B48" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A48)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC48" s="0"/>
@@ -765,8 +776,8 @@
           <t>10.1016/j.intermet.2006.05.016</t>
         </is>
       </c>
-      <c r="B49" s="3">
-        <f>COUNTIF(A:A,"="&amp;A49)</f>
+      <c r="B49" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A49)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC49" s="0"/>
@@ -778,8 +789,8 @@
           <t>10.1016/j.intermet.2006.10.054</t>
         </is>
       </c>
-      <c r="B50" s="3">
-        <f>COUNTIF(A:A,"="&amp;A50)</f>
+      <c r="B50" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A50)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC50" s="0"/>
@@ -791,8 +802,8 @@
           <t>10.1016/j.intermet.2009.03.006</t>
         </is>
       </c>
-      <c r="B51" s="3">
-        <f>COUNTIF(A:A,"="&amp;A51)</f>
+      <c r="B51" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A51)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC51" s="0"/>
@@ -804,8 +815,8 @@
           <t>10.1016/j.intermet.2016.04.006</t>
         </is>
       </c>
-      <c r="B52" s="3">
-        <f>COUNTIF(A:A,"="&amp;A52)</f>
+      <c r="B52" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A52)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC52" s="0"/>
@@ -817,8 +828,8 @@
           <t>10.1016/j.jallcom.2003.09.117</t>
         </is>
       </c>
-      <c r="B53" s="3">
-        <f>COUNTIF(A:A,"="&amp;A53)</f>
+      <c r="B53" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A53)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC53" s="0"/>
@@ -830,8 +841,8 @@
           <t>10.1016/j.jallcom.2006.08.159</t>
         </is>
       </c>
-      <c r="B54" s="3">
-        <f>COUNTIF(A:A,"="&amp;A54)</f>
+      <c r="B54" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A54)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC54" s="0"/>
@@ -843,8 +854,8 @@
           <t>10.1016/j.jallcom.2010.08.019</t>
         </is>
       </c>
-      <c r="B55" s="3">
-        <f>COUNTIF(A:A,"="&amp;A55)</f>
+      <c r="B55" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A55)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC55" s="0"/>
@@ -856,8 +867,8 @@
           <t>10.1016/j.jallcom.2011.02.042</t>
         </is>
       </c>
-      <c r="B56" s="3">
-        <f>COUNTIF(A:A,"="&amp;A56)</f>
+      <c r="B56" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A56)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC56" s="0"/>
@@ -869,8 +880,8 @@
           <t>10.1016/j.jallcom.2011.09.081</t>
         </is>
       </c>
-      <c r="B57" s="3">
-        <f>COUNTIF(A:A,"="&amp;A57)</f>
+      <c r="B57" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A57)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC57" s="0"/>
@@ -882,8 +893,8 @@
           <t>10.1016/j.jallcom.2011.11.035</t>
         </is>
       </c>
-      <c r="B58" s="3">
-        <f>COUNTIF(A:A,"="&amp;A58)</f>
+      <c r="B58" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A58)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC58" s="0"/>
@@ -895,8 +906,8 @@
           <t>10.1016/j.jallcom.2012.10.016</t>
         </is>
       </c>
-      <c r="B59" s="3">
-        <f>COUNTIF(A:A,"="&amp;A59)</f>
+      <c r="B59" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A59)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC59" s="0"/>
@@ -908,8 +919,8 @@
           <t>10.1016/j.jallcom.2013.04.070</t>
         </is>
       </c>
-      <c r="B60" s="3">
-        <f>COUNTIF(A:A,"="&amp;A60)</f>
+      <c r="B60" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A60)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC60" s="0"/>
@@ -921,8 +932,8 @@
           <t>10.1016/j.jallcom.2014.01.173</t>
         </is>
       </c>
-      <c r="B61" s="3">
-        <f>COUNTIF(A:A,"="&amp;A61)</f>
+      <c r="B61" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A61)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC61" s="0"/>
@@ -934,8 +945,8 @@
           <t>10.1016/j.jallcom.2014.02.179</t>
         </is>
       </c>
-      <c r="B62" s="3">
-        <f>COUNTIF(A:A,"="&amp;A62)</f>
+      <c r="B62" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A62)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC62" s="0"/>
@@ -947,8 +958,8 @@
           <t>10.1016/j.jallcom.2014.07.026</t>
         </is>
       </c>
-      <c r="B63" s="3">
-        <f>COUNTIF(A:A,"="&amp;A63)</f>
+      <c r="B63" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A63)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC63" s="0"/>
@@ -960,8 +971,8 @@
           <t>10.1016/j.jallcom.2018.09.139</t>
         </is>
       </c>
-      <c r="B64" s="3">
-        <f>COUNTIF(A:A,"="&amp;A64)</f>
+      <c r="B64" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A64)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC64" s="0"/>
@@ -973,8 +984,8 @@
           <t>10.1016/j.jallcom.2019.02.072</t>
         </is>
       </c>
-      <c r="B65" s="3">
-        <f>COUNTIF(A:A,"="&amp;A65)</f>
+      <c r="B65" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A65)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC65" s="0"/>
@@ -986,8 +997,8 @@
           <t>10.1016/j.jallcom.2019.04.172</t>
         </is>
       </c>
-      <c r="B66" s="3">
-        <f>COUNTIF(A:A,"="&amp;A66)</f>
+      <c r="B66" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A66)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC66" s="0"/>
@@ -999,8 +1010,8 @@
           <t>10.1016/j.jallcom.2019.05.196</t>
         </is>
       </c>
-      <c r="B67" s="3">
-        <f>COUNTIF(A:A,"="&amp;A67)</f>
+      <c r="B67" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A67)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC67" s="0"/>
@@ -1008,22 +1019,22 @@
     </row>
     <row r="68" spans="1:16384" customHeight="1" ht="15.75">
       <c r="A68" s="0" t="s">
-        <v>2</v>
-      </c>
-      <c r="B68" s="3">
-        <f>COUNTIF(A:A,"="&amp;A68)</f>
-        <v>2</v>
+        <v>4</v>
+      </c>
+      <c r="B68" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A68)&gt;1,"yes","no")</f>
+        <v>3</v>
       </c>
       <c r="XFC68" s="0"/>
       <c r="XFD68" s="0"/>
     </row>
     <row r="69" spans="1:16384" customHeight="1" ht="15.75">
       <c r="A69" s="0" t="s">
-        <v>2</v>
-      </c>
-      <c r="B69" s="3">
-        <f>COUNTIF(A:A,"="&amp;A69)</f>
-        <v>2</v>
+        <v>4</v>
+      </c>
+      <c r="B69" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A69)&gt;1,"yes","no")</f>
+        <v>3</v>
       </c>
       <c r="XFC69" s="0"/>
       <c r="XFD69" s="0"/>
@@ -1034,8 +1045,8 @@
           <t>10.1016/j.jallcom.2020.156463</t>
         </is>
       </c>
-      <c r="B70" s="3">
-        <f>COUNTIF(A:A,"="&amp;A70)</f>
+      <c r="B70" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A70)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC70" s="0"/>
@@ -1047,8 +1058,8 @@
           <t>10.1016/j.jmatprotec.2018.07.034</t>
         </is>
       </c>
-      <c r="B71" s="3">
-        <f>COUNTIF(A:A,"="&amp;A71)</f>
+      <c r="B71" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A71)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC71" s="0"/>
@@ -1060,8 +1071,8 @@
           <t>10.1016/j.jmmm.2009.03.067</t>
         </is>
       </c>
-      <c r="B72" s="3">
-        <f>COUNTIF(A:A,"="&amp;A72)</f>
+      <c r="B72" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A72)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC72" s="0"/>
@@ -1073,8 +1084,8 @@
           <t>10.1016/j.jmrt.2018.12.020</t>
         </is>
       </c>
-      <c r="B73" s="3">
-        <f>COUNTIF(A:A,"="&amp;A73)</f>
+      <c r="B73" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A73)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC73" s="0"/>
@@ -1086,8 +1097,8 @@
           <t>10.1016/j.jssc.2012.01.060</t>
         </is>
       </c>
-      <c r="B74" s="3">
-        <f>COUNTIF(A:A,"="&amp;A74)</f>
+      <c r="B74" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A74)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC74" s="0"/>
@@ -1099,8 +1110,8 @@
           <t>10.1016/j.jssc.2012.02.009</t>
         </is>
       </c>
-      <c r="B75" s="3">
-        <f>COUNTIF(A:A,"="&amp;A75)</f>
+      <c r="B75" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A75)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC75" s="0"/>
@@ -1112,8 +1123,8 @@
           <t>10.1016/j.matchar.2005.09.009</t>
         </is>
       </c>
-      <c r="B76" s="3">
-        <f>COUNTIF(A:A,"="&amp;A76)</f>
+      <c r="B76" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A76)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC76" s="0"/>
@@ -1125,8 +1136,8 @@
           <t>10.1016/j.matchar.2005.10.001</t>
         </is>
       </c>
-      <c r="B77" s="3">
-        <f>COUNTIF(A:A,"="&amp;A77)</f>
+      <c r="B77" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A77)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC77" s="0"/>
@@ -1138,8 +1149,8 @@
           <t>10.1016/j.matchar.2006.05.014</t>
         </is>
       </c>
-      <c r="B78" s="3">
-        <f>COUNTIF(A:A,"="&amp;A78)</f>
+      <c r="B78" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A78)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC78" s="0"/>
@@ -1151,8 +1162,8 @@
           <t>10.1016/j.matchar.2006.10.015</t>
         </is>
       </c>
-      <c r="B79" s="3">
-        <f>COUNTIF(A:A,"="&amp;A79)</f>
+      <c r="B79" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A79)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC79" s="0"/>
@@ -1164,8 +1175,8 @@
           <t>10.1016/j.matchar.2006.10.020</t>
         </is>
       </c>
-      <c r="B80" s="3">
-        <f>COUNTIF(A:A,"="&amp;A80)</f>
+      <c r="B80" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A80)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC80" s="0"/>
@@ -1177,8 +1188,8 @@
           <t>10.1016/j.matchar.2008.04.002</t>
         </is>
       </c>
-      <c r="B81" s="3">
-        <f>COUNTIF(A:A,"="&amp;A81)</f>
+      <c r="B81" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A81)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC81" s="0"/>
@@ -1190,8 +1201,8 @@
           <t>10.1016/j.matchar.2012.11.006</t>
         </is>
       </c>
-      <c r="B82" s="3">
-        <f>COUNTIF(A:A,"="&amp;A82)</f>
+      <c r="B82" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A82)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC82" s="0"/>
@@ -1203,8 +1214,8 @@
           <t>10.1016/j.matchemphys.2017.03.037</t>
         </is>
       </c>
-      <c r="B83" s="3">
-        <f>COUNTIF(A:A,"="&amp;A83)</f>
+      <c r="B83" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A83)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC83" s="0"/>
@@ -1216,8 +1227,8 @@
           <t>10.1016/j.matchemphys.2019.01.008</t>
         </is>
       </c>
-      <c r="B84" s="3">
-        <f>COUNTIF(A:A,"="&amp;A84)</f>
+      <c r="B84" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A84)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC84" s="0"/>
@@ -1229,8 +1240,8 @@
           <t>10.1016/j.msea.2006.02.024</t>
         </is>
       </c>
-      <c r="B85" s="3">
-        <f>COUNTIF(A:A,"="&amp;A85)</f>
+      <c r="B85" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A85)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC85" s="0"/>
@@ -1242,8 +1253,8 @@
           <t>10.1016/j.msea.2018.05.078</t>
         </is>
       </c>
-      <c r="B86" s="3">
-        <f>COUNTIF(A:A,"="&amp;A86)</f>
+      <c r="B86" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A86)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC86" s="0"/>
@@ -1255,8 +1266,8 @@
           <t>10.1016/j.msea.2021.141170</t>
         </is>
       </c>
-      <c r="B87" s="3">
-        <f>COUNTIF(A:A,"="&amp;A87)</f>
+      <c r="B87" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A87)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC87" s="0"/>
@@ -1268,8 +1279,8 @@
           <t>10.1016/j.msec.2013.04.015</t>
         </is>
       </c>
-      <c r="B88" s="3">
-        <f>COUNTIF(A:A,"="&amp;A88)</f>
+      <c r="B88" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A88)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC88" s="0"/>
@@ -1281,8 +1292,8 @@
           <t>10.1016/j.mtcomm.2019.100767</t>
         </is>
       </c>
-      <c r="B89" s="3">
-        <f>COUNTIF(A:A,"="&amp;A89)</f>
+      <c r="B89" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A89)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC89" s="0"/>
@@ -1294,8 +1305,8 @@
           <t>10.1016/j.mtcomm.2020.101282</t>
         </is>
       </c>
-      <c r="B90" s="3">
-        <f>COUNTIF(A:A,"="&amp;A90)</f>
+      <c r="B90" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A90)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC90" s="0"/>
@@ -1307,8 +1318,8 @@
           <t>10.1016/j.mtla.2018.11.008</t>
         </is>
       </c>
-      <c r="B91" s="3">
-        <f>COUNTIF(A:A,"="&amp;A91)</f>
+      <c r="B91" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A91)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC91" s="0"/>
@@ -1320,8 +1331,8 @@
           <t>10.1016/j.physleta.2018.02.018</t>
         </is>
       </c>
-      <c r="B92" s="3">
-        <f>COUNTIF(A:A,"="&amp;A92)</f>
+      <c r="B92" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A92)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC92" s="0"/>
@@ -1329,22 +1340,22 @@
     </row>
     <row r="93" spans="1:16384" customHeight="1" ht="15.75">
       <c r="A93" s="0" t="s">
+        <v>5</v>
+      </c>
+      <c r="B93" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A93)&gt;1,"yes","no")</f>
         <v>3</v>
-      </c>
-      <c r="B93" s="3">
-        <f>COUNTIF(A:A,"="&amp;A93)</f>
-        <v>2</v>
       </c>
       <c r="XFC93" s="0"/>
       <c r="XFD93" s="0"/>
     </row>
     <row r="94" spans="1:16384" customHeight="1" ht="15.75">
       <c r="A94" s="0" t="s">
+        <v>5</v>
+      </c>
+      <c r="B94" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A94)&gt;1,"yes","no")</f>
         <v>3</v>
-      </c>
-      <c r="B94" s="3">
-        <f>COUNTIF(A:A,"="&amp;A94)</f>
-        <v>2</v>
       </c>
       <c r="XFC94" s="0"/>
       <c r="XFD94" s="0"/>
@@ -1355,8 +1366,8 @@
           <t>10.1016/j.ssc.2008.12.037</t>
         </is>
       </c>
-      <c r="B95" s="3">
-        <f>COUNTIF(A:A,"="&amp;A95)</f>
+      <c r="B95" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A95)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC95" s="0"/>
@@ -1368,8 +1379,8 @@
           <t>10.1016/j.ssc.2011.07.005</t>
         </is>
       </c>
-      <c r="B96" s="3">
-        <f>COUNTIF(A:A,"="&amp;A96)</f>
+      <c r="B96" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A96)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC96" s="0"/>
@@ -1381,8 +1392,8 @@
           <t>10.1016/j.ssc.2018.08.014</t>
         </is>
       </c>
-      <c r="B97" s="3">
-        <f>COUNTIF(A:A,"="&amp;A97)</f>
+      <c r="B97" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A97)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC97" s="0"/>
@@ -1394,8 +1405,8 @@
           <t>10.1016/j.surfcoat.2020.125675</t>
         </is>
       </c>
-      <c r="B98" s="3">
-        <f>COUNTIF(A:A,"="&amp;A98)</f>
+      <c r="B98" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A98)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC98" s="0"/>
@@ -1407,8 +1418,8 @@
           <t>10.1016/j.surfcoat.2021.126999</t>
         </is>
       </c>
-      <c r="B99" s="3">
-        <f>COUNTIF(A:A,"="&amp;A99)</f>
+      <c r="B99" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A99)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC99" s="0"/>
@@ -1420,8 +1431,8 @@
           <t>10.1016/s0039-9140(02)00471-x</t>
         </is>
       </c>
-      <c r="B100" s="3">
-        <f>COUNTIF(A:A,"="&amp;A100)</f>
+      <c r="B100" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A100)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC100" s="0"/>
@@ -1433,8 +1444,8 @@
           <t>10.1016/s0263-4368(00)00020-2</t>
         </is>
       </c>
-      <c r="B101" s="3">
-        <f>COUNTIF(A:A,"="&amp;A101)</f>
+      <c r="B101" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A101)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC101" s="0"/>
@@ -1446,8 +1457,8 @@
           <t>10.1016/S0263-4368(00)00021-4</t>
         </is>
       </c>
-      <c r="B102" s="3">
-        <f>COUNTIF(A:A,"="&amp;A102)</f>
+      <c r="B102" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A102)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC102" s="0"/>
@@ -1459,8 +1470,8 @@
           <t>10.1016/S0263-4368(99)00002-5</t>
         </is>
       </c>
-      <c r="B103" s="3">
-        <f>COUNTIF(A:A,"="&amp;A103)</f>
+      <c r="B103" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A103)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC103" s="0"/>
@@ -1472,8 +1483,8 @@
           <t>10.1016/s0263-4368(99)00021-9</t>
         </is>
       </c>
-      <c r="B104" s="3">
-        <f>COUNTIF(A:A,"="&amp;A104)</f>
+      <c r="B104" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A104)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC104" s="0"/>
@@ -1485,8 +1496,8 @@
           <t>10.1016/s0921-5093(03)00650-6</t>
         </is>
       </c>
-      <c r="B105" s="3">
-        <f>COUNTIF(A:A,"="&amp;A105)</f>
+      <c r="B105" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A105)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC105" s="0"/>
@@ -1498,8 +1509,8 @@
           <t>10.1016/s0966-9795(02)00125-5</t>
         </is>
       </c>
-      <c r="B106" s="3">
-        <f>COUNTIF(A:A,"="&amp;A106)</f>
+      <c r="B106" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A106)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC106" s="0"/>
@@ -1511,8 +1522,8 @@
           <t>10.1016/s0966-9795(02)00249-2</t>
         </is>
       </c>
-      <c r="B107" s="3">
-        <f>COUNTIF(A:A,"="&amp;A107)</f>
+      <c r="B107" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A107)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC107" s="0"/>
@@ -1524,8 +1535,8 @@
           <t>10.1016/S0966-9795(99)00088-6</t>
         </is>
       </c>
-      <c r="B108" s="3">
-        <f>COUNTIF(A:A,"="&amp;A108)</f>
+      <c r="B108" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A108)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC108" s="0"/>
@@ -1537,8 +1548,8 @@
           <t>10.1016/S1003-6326(18)64867-8</t>
         </is>
       </c>
-      <c r="B109" s="3">
-        <f>COUNTIF(A:A,"="&amp;A109)</f>
+      <c r="B109" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A109)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC109" s="0"/>
@@ -1550,8 +1561,8 @@
           <t>10.1016/s1044-5803(01)00176-0</t>
         </is>
       </c>
-      <c r="B110" s="3">
-        <f>COUNTIF(A:A,"="&amp;A110)</f>
+      <c r="B110" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A110)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC110" s="0"/>
@@ -1563,8 +1574,8 @@
           <t>10.1021/ic401413f</t>
         </is>
       </c>
-      <c r="B111" s="3">
-        <f>COUNTIF(A:A,"="&amp;A111)</f>
+      <c r="B111" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A111)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC111" s="0"/>
@@ -1576,8 +1587,8 @@
           <t>10.1080/00084433.2017.1299907</t>
         </is>
       </c>
-      <c r="B112" s="3">
-        <f>COUNTIF(A:A,"="&amp;A112)</f>
+      <c r="B112" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A112)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC112" s="0"/>
@@ -1589,8 +1600,8 @@
           <t>10.1080/00084433.2017.1409946</t>
         </is>
       </c>
-      <c r="B113" s="3">
-        <f>COUNTIF(A:A,"="&amp;A113)</f>
+      <c r="B113" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A113)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC113" s="0"/>
@@ -1602,8 +1613,8 @@
           <t>10.1088/0953-2048/16/4/317</t>
         </is>
       </c>
-      <c r="B114" s="3">
-        <f>COUNTIF(A:A,"="&amp;A114)</f>
+      <c r="B114" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A114)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC114" s="0"/>
@@ -1615,8 +1626,8 @@
           <t>10.1088/0953-2048/28/9/095016</t>
         </is>
       </c>
-      <c r="B115" s="3">
-        <f>COUNTIF(A:A,"="&amp;A115)</f>
+      <c r="B115" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A115)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC115" s="0"/>
@@ -1628,8 +1639,8 @@
           <t>10.1103/PhysRevB.103.125134</t>
         </is>
       </c>
-      <c r="B116" s="3">
-        <f>COUNTIF(A:A,"="&amp;A116)</f>
+      <c r="B116" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A116)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC116" s="0"/>
@@ -1641,8 +1652,8 @@
           <t>10.1103/PhysRevB.95.094505</t>
         </is>
       </c>
-      <c r="B117" s="3">
-        <f>COUNTIF(A:A,"="&amp;A117)</f>
+      <c r="B117" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A117)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC117" s="0"/>
@@ -1654,8 +1665,8 @@
           <t>10.1103/PhysRevB.95.144505</t>
         </is>
       </c>
-      <c r="B118" s="3">
-        <f>COUNTIF(A:A,"="&amp;A118)</f>
+      <c r="B118" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A118)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC118" s="0"/>
@@ -1667,8 +1678,8 @@
           <t>10.1103/PhysRevB.96.014507</t>
         </is>
       </c>
-      <c r="B119" s="3">
-        <f>COUNTIF(A:A,"="&amp;A119)</f>
+      <c r="B119" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A119)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC119" s="0"/>
@@ -1680,8 +1691,8 @@
           <t>10.1103/physrevb.98.045126</t>
         </is>
       </c>
-      <c r="B120" s="3">
-        <f>COUNTIF(A:A,"="&amp;A120)</f>
+      <c r="B120" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A120)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC120" s="0"/>
@@ -1693,8 +1704,8 @@
           <t>10.1103/PhysRevLett.122.147001</t>
         </is>
       </c>
-      <c r="B121" s="3">
-        <f>COUNTIF(A:A,"="&amp;A121)</f>
+      <c r="B121" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A121)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC121" s="0"/>
@@ -1706,8 +1717,8 @@
           <t>10.1103/physrevmaterials.1.044803</t>
         </is>
       </c>
-      <c r="B122" s="3">
-        <f>COUNTIF(A:A,"="&amp;A122)</f>
+      <c r="B122" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A122)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC122" s="0"/>
@@ -1719,8 +1730,8 @@
           <t>10.1103/PhysRevResearch.2.022001</t>
         </is>
       </c>
-      <c r="B123" s="3">
-        <f>COUNTIF(A:A,"="&amp;A123)</f>
+      <c r="B123" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A123)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC123" s="0"/>
@@ -1732,8 +1743,8 @@
           <t>10.1109/TMAG.2009.2033460</t>
         </is>
       </c>
-      <c r="B124" s="3">
-        <f>COUNTIF(A:A,"="&amp;A124)</f>
+      <c r="B124" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A124)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC124" s="0"/>
@@ -1745,8 +1756,8 @@
           <t>10.1111/j.1525-1594.2008.00546.x</t>
         </is>
       </c>
-      <c r="B125" s="3">
-        <f>COUNTIF(A:A,"="&amp;A125)</f>
+      <c r="B125" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A125)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC125" s="0"/>
@@ -1758,8 +1769,8 @@
           <t>10.1361/105497103770330758</t>
         </is>
       </c>
-      <c r="B126" s="3">
-        <f>COUNTIF(A:A,"="&amp;A126)</f>
+      <c r="B126" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A126)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC126" s="0"/>
@@ -1771,8 +1782,8 @@
           <t>10.1590/1516-1439.329614</t>
         </is>
       </c>
-      <c r="B127" s="3">
-        <f>COUNTIF(A:A,"="&amp;A127)</f>
+      <c r="B127" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A127)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC127" s="0"/>
@@ -1784,8 +1795,8 @@
           <t>10.1590/1516-1439.343514</t>
         </is>
       </c>
-      <c r="B128" s="3">
-        <f>COUNTIF(A:A,"="&amp;A128)</f>
+      <c r="B128" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A128)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC128" s="0"/>
@@ -1797,8 +1808,8 @@
           <t>10.1590/1980-5373-MR-2016-0001</t>
         </is>
       </c>
-      <c r="B129" s="3">
-        <f>COUNTIF(A:A,"="&amp;A129)</f>
+      <c r="B129" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A129)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC129" s="0"/>
@@ -1810,8 +1821,8 @@
           <t>10.1590/1980-5373-mr-2017-0332</t>
         </is>
       </c>
-      <c r="B130" s="3">
-        <f>COUNTIF(A:A,"="&amp;A130)</f>
+      <c r="B130" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A130)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC130" s="0"/>
@@ -1823,8 +1834,8 @@
           <t>10.1590/1980-5373-mr-2017-0468</t>
         </is>
       </c>
-      <c r="B131" s="3">
-        <f>COUNTIF(A:A,"="&amp;A131)</f>
+      <c r="B131" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A131)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC131" s="0"/>
@@ -1836,8 +1847,8 @@
           <t>10.1590/1980-5373-mr-2017-0637</t>
         </is>
       </c>
-      <c r="B132" s="3">
-        <f>COUNTIF(A:A,"="&amp;A132)</f>
+      <c r="B132" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A132)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC132" s="0"/>
@@ -1849,8 +1860,8 @@
           <t>10.1590/1980-5373-mr-2019-0178</t>
         </is>
       </c>
-      <c r="B133" s="3">
-        <f>COUNTIF(A:A,"="&amp;A133)</f>
+      <c r="B133" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A133)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC133" s="0"/>
@@ -1862,8 +1873,8 @@
           <t>10.1590/1980-5373-mr-2019-0305</t>
         </is>
       </c>
-      <c r="B134" s="3">
-        <f>COUNTIF(A:A,"="&amp;A134)</f>
+      <c r="B134" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A134)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC134" s="0"/>
@@ -1875,8 +1886,8 @@
           <t>10.1590/1980-5373-mr-2019-0599</t>
         </is>
       </c>
-      <c r="B135" s="3">
-        <f>COUNTIF(A:A,"="&amp;A135)</f>
+      <c r="B135" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A135)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC135" s="0"/>
@@ -1888,8 +1899,8 @@
           <t>10.1590/s1516-14392010000300009</t>
         </is>
       </c>
-      <c r="B136" s="3">
-        <f>COUNTIF(A:A,"="&amp;A136)</f>
+      <c r="B136" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A136)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC136" s="0"/>
@@ -1901,8 +1912,8 @@
           <t>10.1590/S1516-14392012005000015</t>
         </is>
       </c>
-      <c r="B137" s="3">
-        <f>COUNTIF(A:A,"="&amp;A137)</f>
+      <c r="B137" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A137)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC137" s="0"/>
@@ -1914,8 +1925,8 @@
           <t>10.1590/s1516-14392013005000172</t>
         </is>
       </c>
-      <c r="B138" s="3">
-        <f>COUNTIF(A:A,"="&amp;A138)</f>
+      <c r="B138" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A138)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC138" s="0"/>
@@ -1927,8 +1938,8 @@
           <t>10.1590/s1516-14392014005000018</t>
         </is>
       </c>
-      <c r="B139" s="3">
-        <f>COUNTIF(A:A,"="&amp;A139)</f>
+      <c r="B139" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A139)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC139" s="0"/>
@@ -1940,8 +1951,8 @@
           <t>10.3139/146.111952</t>
         </is>
       </c>
-      <c r="B140" s="3">
-        <f>COUNTIF(A:A,"="&amp;A140)</f>
+      <c r="B140" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A140)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC140" s="0"/>
@@ -1953,8 +1964,8 @@
           <t>10.3390/met8020082</t>
         </is>
       </c>
-      <c r="B141" s="3">
-        <f>COUNTIF(A:A,"="&amp;A141)</f>
+      <c r="B141" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A141)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC141" s="0"/>
@@ -1966,8 +1977,8 @@
           <t>10.3390/met9050589</t>
         </is>
       </c>
-      <c r="B142" s="3">
-        <f>COUNTIF(A:A,"="&amp;A142)</f>
+      <c r="B142" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A142)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC142" s="0"/>
@@ -1979,8 +1990,8 @@
           <t>10.4028/www.scientific.net/jmnm.20-21.139</t>
         </is>
       </c>
-      <c r="B143" s="3">
-        <f>COUNTIF(A:A,"="&amp;A143)</f>
+      <c r="B143" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A143)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC143" s="0"/>
@@ -1992,8 +2003,8 @@
           <t>10.4028/www.scientific.net/jmnm.20-21.145</t>
         </is>
       </c>
-      <c r="B144" s="3">
-        <f>COUNTIF(A:A,"="&amp;A144)</f>
+      <c r="B144" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A144)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC144" s="0"/>
@@ -2005,8 +2016,8 @@
           <t>10.4028/www.scientific.net/JMNM.20-21.201</t>
         </is>
       </c>
-      <c r="B145" s="3">
-        <f>COUNTIF(A:A,"="&amp;A145)</f>
+      <c r="B145" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A145)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC145" s="0"/>
@@ -2018,8 +2029,8 @@
           <t>10.4028/www.scientific.net/MSF.416-418.251</t>
         </is>
       </c>
-      <c r="B146" s="3">
-        <f>COUNTIF(A:A,"="&amp;A146)</f>
+      <c r="B146" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A146)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC146" s="0"/>
@@ -2031,8 +2042,8 @@
           <t>10.4028/www.scientific.net/MSF.660-661.152</t>
         </is>
       </c>
-      <c r="B147" s="3">
-        <f>COUNTIF(A:A,"="&amp;A147)</f>
+      <c r="B147" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A147)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC147" s="0"/>
@@ -2044,8 +2055,8 @@
           <t>10.4028/www.scientific.net/MSF.660-661.405</t>
         </is>
       </c>
-      <c r="B148" s="3">
-        <f>COUNTIF(A:A,"="&amp;A148)</f>
+      <c r="B148" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A148)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC148" s="0"/>
@@ -2057,8 +2068,8 @@
           <t>10.4028/www.scientific.net/msf.802.20</t>
         </is>
       </c>
-      <c r="B149" s="3">
-        <f>COUNTIF(A:A,"="&amp;A149)</f>
+      <c r="B149" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A149)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC149" s="0"/>
@@ -2070,8 +2081,8 @@
           <t>10.4028/www.scientific.net/msf.802.9</t>
         </is>
       </c>
-      <c r="B150" s="3">
-        <f>COUNTIF(A:A,"="&amp;A150)</f>
+      <c r="B150" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A150)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC150" s="0"/>
@@ -2083,8 +2094,8 @@
           <t>10.4028/www.scientific.net/msf.805.199</t>
         </is>
       </c>
-      <c r="B151" s="3">
-        <f>COUNTIF(A:A,"="&amp;A151)</f>
+      <c r="B151" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A151)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC151" s="0"/>
@@ -2096,8 +2107,8 @@
           <t>10.4028/www.scientific.net/MSF.869.952</t>
         </is>
       </c>
-      <c r="B152" s="3">
-        <f>COUNTIF(A:A,"="&amp;A152)</f>
+      <c r="B152" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A152)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC152" s="0"/>
@@ -2109,8 +2120,8 @@
           <t>10.5006/1.3585276</t>
         </is>
       </c>
-      <c r="B153" s="3">
-        <f>COUNTIF(A:A,"="&amp;A153)</f>
+      <c r="B153" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A153)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC153" s="0"/>
@@ -2122,8 +2133,8 @@
           <t>10.5539/jmsr.v9n1p32</t>
         </is>
       </c>
-      <c r="B154" s="3">
-        <f>COUNTIF(A:A,"="&amp;A154)</f>
+      <c r="B154" s="3" t="s">
+        <f>IF(COUNTIF(A:A,"="&amp;A154)&gt;1,"yes","no")</f>
         <v>1</v>
       </c>
       <c r="XFC154" s="0"/>

</xml_diff>